<commit_message>
Actualizacion Diseño e integracion de escaneoPDF
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39ECCE9C-2608-4959-80DF-270760878C84}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D86726-0687-47FF-89A9-23FCDF1B8539}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{07BBAD01-711C-41B6-957E-FFFDE243DC03}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,12 +23,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="109">
   <si>
     <t>CODIGO</t>
   </si>
@@ -288,6 +283,81 @@
   </si>
   <si>
     <t>11</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>37</t>
   </si>
 </sst>
 </file>
@@ -713,10 +783,10 @@
         <v>1771.62</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="F2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -733,7 +803,7 @@
         <v>2137.5100000000002</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
@@ -753,7 +823,7 @@
         <v>2137.5100000000002</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F4" s="1">
         <v>1</v>
@@ -772,8 +842,8 @@
       <c r="D5" s="2">
         <v>2137.5100000000002</v>
       </c>
-      <c r="E5" s="1">
-        <v>10</v>
+      <c r="E5" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
@@ -792,8 +862,8 @@
       <c r="D6" s="1">
         <v>95.5</v>
       </c>
-      <c r="E6" s="1">
-        <v>50</v>
+      <c r="E6" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="F6" s="1">
         <v>1</v>
@@ -812,8 +882,8 @@
       <c r="D7" s="1">
         <v>110.25</v>
       </c>
-      <c r="E7" s="1">
-        <v>40</v>
+      <c r="E7" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="F7" s="1">
         <v>1</v>
@@ -832,8 +902,8 @@
       <c r="D8" s="1">
         <v>620</v>
       </c>
-      <c r="E8" s="1">
-        <v>15</v>
+      <c r="E8" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="F8" s="1">
         <v>1</v>
@@ -872,8 +942,8 @@
       <c r="D10" s="1">
         <v>210.75</v>
       </c>
-      <c r="E10" s="1">
-        <v>25</v>
+      <c r="E10" s="1" t="s">
+        <v>106</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
@@ -892,8 +962,8 @@
       <c r="D11" s="1">
         <v>205.6</v>
       </c>
-      <c r="E11" s="1">
-        <v>20</v>
+      <c r="E11" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="F11" s="1">
         <v>1</v>
@@ -912,8 +982,8 @@
       <c r="D12" s="1">
         <v>205.6</v>
       </c>
-      <c r="E12" s="1">
-        <v>20</v>
+      <c r="E12" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="F12" s="1">
         <v>1</v>
@@ -936,7 +1006,7 @@
         <v>20</v>
       </c>
       <c r="F13" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -952,8 +1022,8 @@
       <c r="D14" s="1">
         <v>120</v>
       </c>
-      <c r="E14" s="1">
-        <v>30</v>
+      <c r="E14" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="F14" s="1">
         <v>1</v>
@@ -972,8 +1042,8 @@
       <c r="D15" s="1">
         <v>180</v>
       </c>
-      <c r="E15" s="1">
-        <v>25</v>
+      <c r="E15" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
@@ -992,8 +1062,8 @@
       <c r="D16" s="2">
         <v>1250</v>
       </c>
-      <c r="E16" s="1">
-        <v>12</v>
+      <c r="E16" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="F16" s="1">
         <v>1</v>
@@ -1012,8 +1082,8 @@
       <c r="D17" s="1">
         <v>220</v>
       </c>
-      <c r="E17" s="1">
-        <v>35</v>
+      <c r="E17" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
@@ -1032,8 +1102,8 @@
       <c r="D18" s="1">
         <v>310</v>
       </c>
-      <c r="E18" s="1">
-        <v>28</v>
+      <c r="E18" s="1" t="s">
+        <v>107</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
@@ -1052,8 +1122,8 @@
       <c r="D19" s="2">
         <v>2850</v>
       </c>
-      <c r="E19" s="1">
-        <v>10</v>
+      <c r="E19" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="F19" s="1">
         <v>1</v>
@@ -1072,8 +1142,8 @@
       <c r="D20" s="1">
         <v>450</v>
       </c>
-      <c r="E20" s="1">
-        <v>22</v>
+      <c r="E20" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="F20" s="1">
         <v>1</v>
@@ -1212,8 +1282,8 @@
       <c r="D27" s="1">
         <v>118.6</v>
       </c>
-      <c r="E27" s="1">
-        <v>120</v>
+      <c r="E27" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="F27" s="1">
         <v>1</v>
@@ -1272,8 +1342,8 @@
       <c r="D30" s="1">
         <v>176.35</v>
       </c>
-      <c r="E30" s="1">
-        <v>40</v>
+      <c r="E30" s="1" t="s">
+        <v>82</v>
       </c>
       <c r="F30" s="1">
         <v>1</v>
@@ -1292,8 +1362,8 @@
       <c r="D31" s="1">
         <v>86.9</v>
       </c>
-      <c r="E31" s="1">
-        <v>75</v>
+      <c r="E31" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="F31" s="1">
         <v>1</v>
@@ -1312,11 +1382,11 @@
       <c r="D32" s="1">
         <v>524.70000000000005</v>
       </c>
-      <c r="E32" s="1">
-        <v>30</v>
+      <c r="E32" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="F32" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1352,8 +1422,8 @@
       <c r="D34" s="1">
         <v>63.25</v>
       </c>
-      <c r="E34" s="1">
-        <v>80</v>
+      <c r="E34" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="F34" s="1">
         <v>1</v>
@@ -1392,8 +1462,8 @@
       <c r="D36" s="1">
         <v>3249</v>
       </c>
-      <c r="E36" s="1">
-        <v>12</v>
+      <c r="E36" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
@@ -1416,7 +1486,7 @@
         <v>28</v>
       </c>
       <c r="F37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reparacion del boton de monto abonado
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D86726-0687-47FF-89A9-23FCDF1B8539}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47401D2F-2CF3-4BB1-93B8-C929FAAB5C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{07BBAD01-711C-41B6-957E-FFFDE243DC03}"/>
+    <workbookView xWindow="3024" yWindow="2304" windowWidth="16740" windowHeight="9372" xr2:uid="{07BBAD01-711C-41B6-957E-FFFDE243DC03}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="122">
   <si>
     <t>CODIGO</t>
   </si>
@@ -282,24 +282,9 @@
     <t>41</t>
   </si>
   <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
-    <t>42</t>
-  </si>
-  <si>
     <t>31</t>
   </si>
   <si>
@@ -315,106 +300,103 @@
     <t>81</t>
   </si>
   <si>
-    <t>43</t>
+    <t>32</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>CATEGORIA</t>
+  </si>
+  <si>
+    <t>MARCA</t>
+  </si>
+  <si>
+    <t>STOCK_MINIMO</t>
+  </si>
+  <si>
+    <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>IMAGEN_RUTA</t>
+  </si>
+  <si>
+    <t>1,771.62</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\IMAGENES\W2300A.jpg</t>
+  </si>
+  <si>
+    <t>Consumibles</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>47</t>
   </si>
   <si>
     <t>21</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>52</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>121</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>53</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>CATEGORIA</t>
-  </si>
-  <si>
-    <t>MARCA</t>
-  </si>
-  <si>
-    <t>STOCK_MINIMO</t>
-  </si>
-  <si>
-    <t>OBSERVACIONES</t>
-  </si>
-  <si>
-    <t>IMAGEN_RUTA</t>
-  </si>
-  <si>
-    <t>1,771.62</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>54</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\IMAGENES\W2300A.jpg</t>
-  </si>
-  <si>
-    <t>Consumibles</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>0</t>
   </si>
 </sst>
 </file>
@@ -422,7 +404,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,15 +433,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -797,16 +776,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{877AF9B0-D8EB-40CB-AC5E-6B8E2D94635F}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="1" width="10.8984375" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="124.19921875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="10.88671875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="124.21875" collapsed="true"/>
     <col min="3" max="3" bestFit="true" customWidth="true" style="1" width="14.0" collapsed="true"/>
     <col min="4" max="4" bestFit="true" customWidth="true" style="1" width="15.0" collapsed="true"/>
-    <col min="5" max="5" style="1" width="10.8984375" collapsed="true"/>
+    <col min="5" max="5" style="1" width="10.88671875" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" width="19.77734375" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -826,22 +806,22 @@
         <v>48</v>
       </c>
       <c r="G1" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="H1" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="I1" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="J1" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="K1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -852,31 +832,31 @@
         <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>127</v>
+        <v>104</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="G2" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="H2" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="I2" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="J2" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="K2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -890,13 +870,13 @@
         <v>2137.5100000000002</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -910,13 +890,13 @@
         <v>2137.5100000000002</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>121</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -930,13 +910,13 @@
         <v>2137.5100000000002</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -950,13 +930,13 @@
         <v>95.5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F6" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -970,13 +950,13 @@
         <v>110.25</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="F7" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -996,7 +976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1016,7 +996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
@@ -1030,13 +1010,13 @@
         <v>210.75</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>123</v>
+        <v>84</v>
       </c>
       <c r="F10" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -1056,7 +1036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -1070,13 +1050,13 @@
         <v>205.6</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F12" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
@@ -1096,7 +1076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
@@ -1110,13 +1090,13 @@
         <v>120</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F14" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -1130,13 +1110,13 @@
         <v>180</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>34</v>
       </c>
@@ -1150,13 +1130,13 @@
         <v>1250</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F16" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>36</v>
       </c>
@@ -1170,13 +1150,13 @@
         <v>220</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
@@ -1190,13 +1170,13 @@
         <v>310</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1210,13 +1190,13 @@
         <v>2850</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F19" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>42</v>
       </c>
@@ -1230,13 +1210,13 @@
         <v>450</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F20" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>44</v>
       </c>
@@ -1256,7 +1236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>46</v>
       </c>
@@ -1276,7 +1256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>51</v>
       </c>
@@ -1296,7 +1276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
@@ -1316,7 +1296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>55</v>
       </c>
@@ -1336,7 +1316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>57</v>
       </c>
@@ -1356,7 +1336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>59</v>
       </c>
@@ -1370,13 +1350,13 @@
         <v>118.6</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F27" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>61</v>
       </c>
@@ -1396,7 +1376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>63</v>
       </c>
@@ -1416,7 +1396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
@@ -1436,7 +1416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
@@ -1450,13 +1430,13 @@
         <v>86.9</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="F31" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>69</v>
       </c>
@@ -1470,13 +1450,13 @@
         <v>524.70000000000005</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F32" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
@@ -1496,7 +1476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>73</v>
       </c>
@@ -1510,13 +1490,13 @@
         <v>63.25</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F34" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>76</v>
       </c>
@@ -1536,7 +1516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>78</v>
       </c>
@@ -1550,13 +1530,13 @@
         <v>3249</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F36" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>80</v>
       </c>

</xml_diff>